<commit_message>
feat: improve training exams and employee workflows
</commit_message>
<xml_diff>
--- a/backend/src/main/resources/templates/question-bank-template.xlsx
+++ b/backend/src/main/resources/templates/question-bank-template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="题库导入" sheetId="1" r:id="R1785fcb335204011"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写示例与说明" sheetId="2" r:id="R7754636b63414433"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="题库导入" sheetId="1" r:id="R049aab95558e43ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="填写示例与说明" sheetId="2" r:id="Rec0d3e0343b54665"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14621,7 +14621,7 @@
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="34" t="str">
-        <x:v>2  题型、默认分值必须填写；题干和正确答案不能为空。</x:v>
+        <x:v>2  题型必须填写；默认分值可选填；题干和正确答案不能为空。</x:v>
       </x:c>
       <x:c r="B7" s="34"/>
       <x:c r="C7" s="34"/>
@@ -14848,10 +14848,10 @@
         <x:v>默认分值</x:v>
       </x:c>
       <x:c r="B20" s="41" t="str">
-        <x:v>必填</x:v>
+        <x:v>选填</x:v>
       </x:c>
       <x:c r="C20" s="41" t="str">
-        <x:v>必须是大于 0 的数字，最多保留两位小数</x:v>
+        <x:v>可填写大于 0 的数字，最多保留两位小数；留空时可在组卷时设置</x:v>
       </x:c>
       <x:c r="D20" s="41"/>
       <x:c r="E20" s="41"/>
@@ -14859,7 +14859,7 @@
       <x:c r="G20" s="41"/>
       <x:c r="H20" s="41"/>
       <x:c r="I20" s="41" t="str">
-        <x:v>5 或 2.5</x:v>
+        <x:v>留空、5 或 2.5</x:v>
       </x:c>
       <x:c r="J20" s="41"/>
       <x:c r="K20" s="41"/>
@@ -15088,9 +15088,7 @@
       <x:c r="J31" s="48" t="str">
         <x:v>工作账号不得外借。</x:v>
       </x:c>
-      <x:c r="K31" s="48" t="n">
-        <x:v>5</x:v>
-      </x:c>
+      <x:c r="K31" s="48"/>
       <x:c r="L31" s="48" t="str">
         <x:v>安全管理</x:v>
       </x:c>

</xml_diff>